<commit_message>
feat: 合并溢价率过滤 (check_premium + NAV加载)
- 加载38只ETF净值数据，判断溢价率>20%则过滤
- filtered 新增 premium_filtered 字段
- 卖出理由新增溢价率过滤原因
- 已生效: 中韩半导体ETF被溢价率过滤剔除
</commit_message>
<xml_diff>
--- a/backtest/results_172/七星172_交易记录_2026.xlsx
+++ b/backtest/results_172/七星172_交易记录_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2496,6 +2496,72 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>科创50ETF易方达</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>sh588080</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>卖出</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1.822</v>
+      </c>
+      <c r="F65" t="n">
+        <v>11.2327</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>盈利保护(回撤超5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>创业板成长ETF华夏</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>sz159967</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F66" t="n">
+        <v>5.0321</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>动量排名第1/38</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>